<commit_message>
add code that creates overview of scores file
</commit_message>
<xml_diff>
--- a/data/raw/metamethod review/master coding/monotonic_scores.xlsx
+++ b/data/raw/metamethod review/master coding/monotonic_scores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/308fe5676bbb12c4/Documents/GitHub/igt-project/data/raw/metamethod review/master coding/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="34" documentId="11_EE7FFDCE8F79A8D366075C52F3B782B6345FCE38" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F41F4381-ACCB-4702-9CBA-DA799B3A744E}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="11_EE7FFDCE8F79A8D366075C52F3B782B6345FCE38" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D220EA51-0A6A-4D3D-A3AB-7A4F8E41833B}"/>
   <bookViews>
-    <workbookView xWindow="31935" yWindow="0" windowWidth="17160" windowHeight="19740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="48735" yWindow="735" windowWidth="38700" windowHeight="15105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -98,10 +98,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -392,9 +388,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B44"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -402,7 +398,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>1007</v>
       </c>
@@ -410,7 +406,7 @@
         <v>1065</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>1047</v>
       </c>
@@ -418,7 +414,7 @@
         <v>1001</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>1048</v>
       </c>
@@ -426,7 +422,7 @@
         <v>1002</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>1049</v>
       </c>
@@ -434,7 +430,7 @@
         <v>1003</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>1050</v>
       </c>
@@ -442,7 +438,7 @@
         <v>1004</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>1051</v>
       </c>
@@ -450,7 +446,7 @@
         <v>1005</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>1052</v>
       </c>
@@ -458,7 +454,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>1056</v>
       </c>
@@ -466,7 +462,7 @@
         <v>1001</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>1057</v>
       </c>
@@ -474,7 +470,7 @@
         <v>1002</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>1058</v>
       </c>
@@ -482,7 +478,7 @@
         <v>1003</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A12">
         <v>1059</v>
       </c>
@@ -490,7 +486,7 @@
         <v>1004</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A13">
         <v>1060</v>
       </c>
@@ -498,7 +494,7 @@
         <v>1005</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A14">
         <v>1061</v>
       </c>
@@ -506,7 +502,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>1067</v>
       </c>
@@ -514,7 +510,7 @@
         <v>1066</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A16">
         <v>2001</v>
       </c>
@@ -522,7 +518,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A17">
         <v>2002</v>
       </c>
@@ -530,7 +526,7 @@
         <v>1055</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A18">
         <v>2007</v>
       </c>
@@ -538,7 +534,7 @@
         <v>1062</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A19">
         <v>2008</v>
       </c>
@@ -546,7 +542,7 @@
         <v>1063</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A20">
         <v>2009</v>
       </c>
@@ -554,7 +550,7 @@
         <v>1064</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A21">
         <v>2031</v>
       </c>
@@ -562,7 +558,7 @@
         <v>1001</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A22">
         <v>2089</v>
       </c>
@@ -570,7 +566,7 @@
         <v>1062</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A23">
         <v>2090</v>
       </c>
@@ -578,7 +574,7 @@
         <v>1063</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A24">
         <v>2091</v>
       </c>
@@ -586,7 +582,7 @@
         <v>1064</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A25">
         <v>2092</v>
       </c>
@@ -594,7 +590,7 @@
         <v>1065</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A26">
         <v>2095</v>
       </c>
@@ -602,7 +598,7 @@
         <v>2098</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A27">
         <v>2096</v>
       </c>
@@ -610,7 +606,7 @@
         <v>2099</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A28">
         <v>2097</v>
       </c>
@@ -618,7 +614,7 @@
         <v>2100</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A29">
         <v>2098</v>
       </c>
@@ -626,7 +622,7 @@
         <v>2095</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A30">
         <v>2099</v>
       </c>
@@ -634,7 +630,7 @@
         <v>2096</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A31">
         <v>2100</v>
       </c>
@@ -642,7 +638,7 @@
         <v>2097</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A32">
         <v>4017</v>
       </c>
@@ -650,7 +646,7 @@
         <v>4016</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A33" s="2">
         <v>3003</v>
       </c>
@@ -658,7 +654,7 @@
         <v>4016</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A34" s="2">
         <v>3007</v>
       </c>
@@ -666,7 +662,7 @@
         <v>4016</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A35" s="2">
         <v>3009</v>
       </c>
@@ -674,7 +670,7 @@
         <v>4016</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A36" s="2">
         <v>3012</v>
       </c>
@@ -682,7 +678,7 @@
         <v>4016</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A37" s="2">
         <v>3020</v>
       </c>
@@ -690,7 +686,7 @@
         <v>4016</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A38" s="2">
         <v>3004</v>
       </c>
@@ -698,7 +694,7 @@
         <v>4016</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A39" s="2">
         <v>3019</v>
       </c>
@@ -706,7 +702,7 @@
         <v>4016</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A40" s="2">
         <v>3033</v>
       </c>
@@ -714,7 +710,7 @@
         <v>4016</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A41" s="2">
         <v>3010</v>
       </c>
@@ -722,15 +718,15 @@
         <v>3025</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A42" s="2">
+        <v>3027</v>
+      </c>
+      <c r="B42">
         <v>3005</v>
       </c>
-      <c r="B42">
-        <v>3027</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A43" s="2">
         <v>4001</v>
       </c>
@@ -738,7 +734,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A44" s="2">
         <v>4002</v>
       </c>

</xml_diff>